<commit_message>
Harden Ghana bank parsers and add unified go-live verification.
Refresh NIB/GCB/Prudential/Absa/BOA/SCB parse paths against specimen outputs, and ship a single verify script covering matching, identity, parsers, and optional live API smoke.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/corrected-bank-specimens-for-user/02-nib/parsed-excel/NIB(1102037505201)[10535] - parsed.xlsx
+++ b/corrected-bank-specimens-for-user/02-nib/parsed-excel/NIB(1102037505201)[10535] - parsed.xlsx
@@ -32,11 +32,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -428,7 +425,7 @@
         <v>Exported</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-07-17T19:29:57.516Z</v>
+        <v>2026-08-10T12:09:43.382Z</v>
       </c>
     </row>
     <row r="5">
@@ -486,7 +483,7 @@
         <v>TT23278G3SMB</v>
       </c>
       <c r="C10" t="str">
-        <v>Cash Deposit</v>
+        <v>Cash Deposit DARKO FRANKLIN A</v>
       </c>
       <c r="D10" t="str">
         <v>05/10/2023</v>
@@ -506,7 +503,7 @@
         <v>FT23278B7PSK</v>
       </c>
       <c r="C11" t="str">
-        <v>Inward Cheque - Dr</v>
+        <v>Inward Cheque - Dr CHQ NO 000399 FROM NIB ACCRA MAIN IFO Chq 000399 ifo Ordering Cust: 375052</v>
       </c>
       <c r="D11" t="str">
         <v>05/10/2023</v>
@@ -526,7 +523,7 @@
         <v>TT232794G1HG</v>
       </c>
       <c r="C12" t="str">
-        <v>Cash Withdrawal</v>
+        <v>Cash Withdrawal ISAAC YAW NORTEY By cheque No: 000404</v>
       </c>
       <c r="D12" t="str">
         <v>06/10/2023</v>
@@ -546,7 +543,7 @@
         <v>TT23289B7W4M</v>
       </c>
       <c r="C13" t="str">
-        <v>Cash Deposit</v>
+        <v>Cash Deposit ADELAIDE AGYEMANG</v>
       </c>
       <c r="D13" t="str">
         <v>16/10/2023</v>
@@ -566,7 +563,7 @@
         <v>FT232908N9FV</v>
       </c>
       <c r="C14" t="str">
-        <v>Inward Cheque - Dr</v>
+        <v>Inward Cheque - Dr CHQ NO 000376 FROM NIB ACCRA MAIN IFO Chq 000376 ifo FALIDU TAHIRU Ordering Cust: 375052</v>
       </c>
       <c r="D14" t="str">
         <v>17/10/2023</v>
@@ -586,7 +583,7 @@
         <v>FT232916PM3C</v>
       </c>
       <c r="C15" t="str">
-        <v>BN K Inward Telex Paym ent 18 OCT 23</v>
+        <v>Inward Telex Payment GHANA COCOA Ordering Cust:</v>
       </c>
       <c r="D15" t="str">
         <v>18/10/2023</v>
@@ -606,7 +603,7 @@
         <v>FT23291WT4P5</v>
       </c>
       <c r="C16" t="str">
-        <v>BN K Inward Telex Paym ent 18 OCT 23</v>
+        <v>Inward Telex Payment GHANA COCOA Ordering Cust:</v>
       </c>
       <c r="D16" t="str">
         <v>18/10/2023</v>
@@ -626,7 +623,7 @@
         <v>FT23291CY4ZQ</v>
       </c>
       <c r="C17" t="str">
-        <v>BN K Inward Telex Paym ent 18 OCT 23</v>
+        <v>Inward Telex Payment GHANA COCOA Ordering Cust:</v>
       </c>
       <c r="D17" t="str">
         <v>18/10/2023</v>
@@ -646,7 +643,7 @@
         <v>TT23292CMJXC</v>
       </c>
       <c r="C18" t="str">
-        <v>Cash Withdrawal</v>
+        <v>Cash Withdrawal OBIRI SAMUEL By cheque No: 000370</v>
       </c>
       <c r="D18" t="str">
         <v>19/10/2023</v>
@@ -666,7 +663,7 @@
         <v>FT23296QM2M2</v>
       </c>
       <c r="C19" t="str">
-        <v>Inward Cheque - Dr</v>
+        <v>Inward Cheque - Dr CHQ NO 000403 FROM NIB ACCRA MAIN IFO Chq 000403 ifo Ordering Cust: 375052</v>
       </c>
       <c r="D19" t="str">
         <v>23/10/2023</v>
@@ -686,7 +683,7 @@
         <v>TT233039NSWX</v>
       </c>
       <c r="C20" t="str">
-        <v>Cash Withdrawal</v>
+        <v>Cash Withdrawal ABEM KENNEDY By cheque No: 000407</v>
       </c>
       <c r="D20" t="str">
         <v>30/10/2023</v>
@@ -706,7 +703,7 @@
         <v>FT23304393BV</v>
       </c>
       <c r="C21" t="str">
-        <v>Application Of Char ges</v>
+        <v>Application Of Charges ACCT MAINT CHARGE AS AT 31 OCT 2023</v>
       </c>
       <c r="D21" t="str">
         <v>31/10/2023</v>

</xml_diff>